<commit_message>
feat: refactor iivw_diagnose, expand QA suite, and bump versions
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_regtab_models.xlsx
+++ b/tabtools/demo/demo_regtab_models.xlsx
@@ -405,10 +405,10 @@
     <t>GLM Poisson</t>
   </si>
   <si>
-    <t>3.29</t>
+    <t>49369.13</t>
   </si>
   <si>
-    <t>-127065.63</t>
+    <t>49414.83</t>
   </si>
   <si>
     <t>(-0.02, 0.02)</t>
@@ -41081,7 +41081,7 @@
   <cols>
     <col min="1" max="1" width="1.7109375" style="1285" customWidth="true"/>
     <col min="2" max="2" width="28.7109375" style="1286" customWidth="true"/>
-    <col min="3" max="3" width="10.2109375" style="1287" customWidth="true"/>
+    <col min="3" max="3" width="8.2109375" style="1287" customWidth="true"/>
     <col min="4" max="4" width="13.2109375" style="1288" customWidth="true"/>
     <col min="5" max="5" width="7.7109375" style="1289" customWidth="true"/>
   </cols>

</xml_diff>

<commit_message>
finegray: add optimizer/tie-handling; gcomp: expand QA audit suite
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_regtab_models.xlsx
+++ b/tabtools/demo/demo_regtab_models.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="636" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="636" uniqueCount="206">
   <si>
     <t>Table 5h. Multinomial Logit -- Education Level</t>
   </si>
@@ -393,6 +393,9 @@
     <t>0.81</t>
   </si>
   <si>
+    <t>&gt;0.99</t>
+  </si>
+  <si>
     <t>0.82</t>
   </si>
   <si>
@@ -409,15 +412,6 @@
   </si>
   <si>
     <t>49414.83</t>
-  </si>
-  <si>
-    <t>(-0.02, 0.02)</t>
-  </si>
-  <si>
-    <t>(-0.00, 0.00)</t>
-  </si>
-  <si>
-    <t>(-0.02, 0.03)</t>
   </si>
   <si>
     <t>Table 5n. Panel Random-Effects Regression</t>
@@ -39911,7 +39905,7 @@
   <sheetData>
     <row r="1" s="2220" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="2298" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B1" s="2290" t="s">
         <v>1</v>
@@ -39934,7 +39928,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2328" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D2" s="2329" t="s">
         <v>1</v>
@@ -39965,13 +39959,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="2362" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C4" s="2408" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D4" s="2409" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E4" s="2410" t="s">
         <v>74</v>
@@ -39982,13 +39976,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="2363" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2411" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D5" s="2412" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E5" s="2413" t="s">
         <v>74</v>
@@ -40002,7 +39996,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="2414" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D6" s="2415" t="s">
         <v>1</v>
@@ -40019,7 +40013,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="2417" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D7" s="2418" t="s">
         <v>1</v>
@@ -40036,7 +40030,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="2420" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D8" s="2421" t="s">
         <v>1</v>
@@ -40053,7 +40047,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="2423" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D9" s="2424" t="s">
         <v>1</v>
@@ -40070,7 +40064,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="2426" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D10" s="2427" t="s">
         <v>1</v>
@@ -40957,7 +40951,7 @@
         <v>119</v>
       </c>
       <c r="E6" s="1265" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -40974,7 +40968,7 @@
         <v>120</v>
       </c>
       <c r="E7" s="1268" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8">
@@ -40991,7 +40985,7 @@
         <v>120</v>
       </c>
       <c r="E8" s="1271" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
@@ -41082,13 +41076,13 @@
     <col min="1" max="1" width="1.7109375" style="1285" customWidth="true"/>
     <col min="2" max="2" width="28.7109375" style="1286" customWidth="true"/>
     <col min="3" max="3" width="8.2109375" style="1287" customWidth="true"/>
-    <col min="4" max="4" width="13.2109375" style="1288" customWidth="true"/>
+    <col min="4" max="4" width="12.2109375" style="1288" customWidth="true"/>
     <col min="5" max="5" width="7.7109375" style="1289" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" s="1284" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="1369" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1361" t="s">
         <v>1</v>
@@ -41111,7 +41105,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1400" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D2" s="1401" t="s">
         <v>1</v>
@@ -41145,10 +41139,10 @@
         <v>46</v>
       </c>
       <c r="C4" s="1469" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1470" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="E4" s="1471" t="s">
         <v>121</v>
@@ -41162,10 +41156,10 @@
         <v>47</v>
       </c>
       <c r="C5" s="1472" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="D5" s="1473" t="s">
-        <v>130</v>
+        <v>29</v>
       </c>
       <c r="E5" s="1474" t="s">
         <v>122</v>
@@ -41179,13 +41173,13 @@
         <v>48</v>
       </c>
       <c r="C6" s="1475" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="D6" s="1476" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="E6" s="1477" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -41196,13 +41190,13 @@
         <v>49</v>
       </c>
       <c r="C7" s="1478" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="D7" s="1479" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="E7" s="1480" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8">
@@ -41213,13 +41207,13 @@
         <v>50</v>
       </c>
       <c r="C8" s="1481" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="D8" s="1482" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="E8" s="1483" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
@@ -41247,7 +41241,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="1487" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D10" s="1488" t="s">
         <v>1</v>
@@ -41264,7 +41258,7 @@
         <v>12</v>
       </c>
       <c r="C11" s="1490" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D11" s="1491" t="s">
         <v>1</v>
@@ -41298,7 +41292,7 @@
   <sheetData>
     <row r="1" s="1493" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="1557" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1549" t="s">
         <v>1</v>
@@ -41321,7 +41315,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1585" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D2" s="1586" t="s">
         <v>1</v>
@@ -41352,13 +41346,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="1615" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C4" s="1638" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D4" s="1639" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E4" s="1640" t="s">
         <v>74</v>
@@ -41369,13 +41363,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="1616" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C5" s="1641" t="s">
         <v>77</v>
       </c>
       <c r="D5" s="1642" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E5" s="1643" t="s">
         <v>74</v>
@@ -41389,10 +41383,10 @@
         <v>51</v>
       </c>
       <c r="C6" s="1644" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D6" s="1645" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E6" s="1646" t="s">
         <v>74</v>
@@ -41406,7 +41400,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="1647" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D7" s="1648" t="s">
         <v>1</v>
@@ -41420,10 +41414,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="1631" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C8" s="1650" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D8" s="1651" t="s">
         <v>1</v>
@@ -41456,7 +41450,7 @@
   <sheetData>
     <row r="1" s="1653" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="1738" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1730" t="s">
         <v>1</v>
@@ -41479,7 +41473,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1769" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D2" s="1770" t="s">
         <v>1</v>
@@ -41513,13 +41507,13 @@
         <v>46</v>
       </c>
       <c r="C4" s="1831" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D4" s="1832" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E4" s="1833" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5">
@@ -41536,7 +41530,7 @@
         <v>64</v>
       </c>
       <c r="E5" s="1836" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6">
@@ -41550,10 +41544,10 @@
         <v>57</v>
       </c>
       <c r="D6" s="1838" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E6" s="1839" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7">
@@ -41564,13 +41558,13 @@
         <v>49</v>
       </c>
       <c r="C7" s="1840" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D7" s="1841" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E7" s="1842" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8">
@@ -41581,13 +41575,13 @@
         <v>50</v>
       </c>
       <c r="C8" s="1843" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D8" s="1844" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E8" s="1845" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9">
@@ -41598,10 +41592,10 @@
         <v>51</v>
       </c>
       <c r="C9" s="1846" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D9" s="1847" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E9" s="1848" t="s">
         <v>74</v>
@@ -41668,7 +41662,7 @@
   <sheetData>
     <row r="1" s="1855" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="1989" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B1" s="1978" t="s">
         <v>1</v>
@@ -41700,7 +41694,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2048" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D2" s="2049" t="s">
         <v>1</v>
@@ -41709,7 +41703,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="2051" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G2" s="2052" t="s">
         <v>1</v>
@@ -41749,25 +41743,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="2098" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C4" s="2166" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D4" s="2167" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E4" s="2168" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F4" s="2169" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G4" s="2170" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H4" s="2171" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5">
@@ -41775,22 +41769,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="2099" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C5" s="2172" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D5" s="2173" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E5" s="2174" t="s">
         <v>74</v>
       </c>
       <c r="F5" s="2175" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G5" s="2176" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H5" s="2177" t="s">
         <v>74</v>
@@ -41801,22 +41795,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="2100" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C6" s="2178" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D6" s="2179" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E6" s="2180" t="s">
         <v>74</v>
       </c>
       <c r="F6" s="2181" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G6" s="2182" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H6" s="2183" t="s">
         <v>74</v>
@@ -41827,22 +41821,22 @@
         <v>1</v>
       </c>
       <c r="B7" s="2101" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C7" s="2184" t="s">
         <v>43</v>
       </c>
       <c r="D7" s="2185" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E7" s="2186" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F7" s="2187" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G7" s="2188" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H7" s="2189" t="s">
         <v>92</v>
@@ -41853,22 +41847,22 @@
         <v>1</v>
       </c>
       <c r="B8" s="2102" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C8" s="2190" t="s">
         <v>40</v>
       </c>
       <c r="D8" s="2191" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E8" s="2192" t="s">
         <v>74</v>
       </c>
       <c r="F8" s="2193" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G8" s="2194" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H8" s="2195" t="s">
         <v>74</v>
@@ -41882,7 +41876,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="2196" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D9" s="2197" t="s">
         <v>1</v>
@@ -41891,7 +41885,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="2199" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G9" s="2200" t="s">
         <v>1</v>
@@ -41908,7 +41902,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="2202" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D10" s="2203" t="s">
         <v>1</v>
@@ -41917,7 +41911,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="2205" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G10" s="2206" t="s">
         <v>1</v>
@@ -41934,7 +41928,7 @@
         <v>12</v>
       </c>
       <c r="C11" s="2208" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D11" s="2209" t="s">
         <v>1</v>
@@ -41943,7 +41937,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="2211" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G11" s="2212" t="s">
         <v>1</v>
@@ -41960,7 +41954,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="2214" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D12" s="2215" t="s">
         <v>1</v>
@@ -41969,7 +41963,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="2217" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G12" s="2218" t="s">
         <v>1</v>

</xml_diff>